<commit_message>
fix: hysteresis shading, label collision, axis limits; close reference loop
</commit_message>
<xml_diff>
--- a/examples/reference_mesoporous.xlsx
+++ b/examples/reference_mesoporous.xlsx
@@ -441,7 +441,7 @@
         <v>0.0004999999999999999</v>
       </c>
       <c r="G2" t="n">
-        <v>2.303859961664848</v>
+        <v>2.30747084272073</v>
       </c>
     </row>
     <row r="3">
@@ -449,7 +449,7 @@
         <v>0.0006667607160816619</v>
       </c>
       <c r="G3" t="n">
-        <v>3.016264418083535</v>
+        <v>3.020991863426574</v>
       </c>
     </row>
     <row r="4">
@@ -457,7 +457,7 @@
         <v>0.0008891397050194613</v>
       </c>
       <c r="G4" t="n">
-        <v>3.926870476933046</v>
+        <v>3.933025131491047</v>
       </c>
     </row>
     <row r="5">
@@ -465,7 +465,7 @@
         <v>0.001185686852830827</v>
       </c>
       <c r="G5" t="n">
-        <v>5.076128606621731</v>
+        <v>5.084084514067436</v>
       </c>
     </row>
     <row r="6">
@@ -473,7 +473,7 @@
         <v>0.001581138830084189</v>
       </c>
       <c r="G6" t="n">
-        <v>6.503599212612918</v>
+        <v>6.513792420352377</v>
       </c>
     </row>
     <row r="7">
@@ -481,7 +481,7 @@
         <v>0.002108482517142911</v>
       </c>
       <c r="G7" t="n">
-        <v>8.241962667316397</v>
+        <v>8.254880443289723</v>
       </c>
     </row>
     <row r="8">
@@ -489,7 +489,7 @@
         <v>0.002811706625951745</v>
       </c>
       <c r="G8" t="n">
-        <v>10.30893482581215</v>
+        <v>10.325092204337</v>
       </c>
     </row>
     <row r="9">
@@ -497,7 +497,7 @@
         <v>0.003749471046662279</v>
       </c>
       <c r="G9" t="n">
-        <v>12.69833564220343</v>
+        <v>12.71823797150062</v>
       </c>
     </row>
     <row r="10">
@@ -505,7 +505,7 @@
         <v>0.004999999999999999</v>
       </c>
       <c r="G10" t="n">
-        <v>15.37290943475505</v>
+        <v>15.39700367154695</v>
       </c>
     </row>
     <row r="11">
@@ -513,7 +513,7 @@
         <v>0.006667607160816619</v>
       </c>
       <c r="G11" t="n">
-        <v>18.26236905522654</v>
+        <v>18.29099199392694</v>
       </c>
     </row>
     <row r="12">
@@ -521,7 +521,7 @@
         <v>0.008891397050194613</v>
       </c>
       <c r="G12" t="n">
-        <v>21.26949262756624</v>
+        <v>21.30282868499813</v>
       </c>
     </row>
     <row r="13">
@@ -529,7 +529,7 @@
         <v>0.01185686852830828</v>
       </c>
       <c r="G13" t="n">
-        <v>24.28447117561458</v>
+        <v>24.32253266302234</v>
       </c>
     </row>
     <row r="14">
@@ -537,7 +537,7 @@
         <v>0.0158113883008419</v>
       </c>
       <c r="G14" t="n">
-        <v>27.20411216107202</v>
+        <v>27.24674965418316</v>
       </c>
     </row>
     <row r="15">
@@ -545,7 +545,7 @@
         <v>0.02108482517142911</v>
       </c>
       <c r="G15" t="n">
-        <v>29.95020157661082</v>
+        <v>29.99714306493577</v>
       </c>
     </row>
     <row r="16">
@@ -553,7 +553,7 @@
         <v>0.02811706625951745</v>
       </c>
       <c r="G16" t="n">
-        <v>32.48202269827544</v>
+        <v>32.53293235527264</v>
       </c>
     </row>
     <row r="17">
@@ -561,7 +561,7 @@
         <v>0.03749471046662279</v>
       </c>
       <c r="G17" t="n">
-        <v>34.80128732386256</v>
+        <v>34.8558320059218</v>
       </c>
     </row>
     <row r="18">
@@ -569,7 +569,7 @@
         <v>0.05</v>
       </c>
       <c r="G18" t="n">
-        <v>36.95144485625146</v>
+        <v>37.00935951879131</v>
       </c>
     </row>
     <row r="19">
@@ -577,7 +577,7 @@
         <v>0.07142857142857142</v>
       </c>
       <c r="G19" t="n">
-        <v>39.50961954499967</v>
+        <v>39.57154368062943</v>
       </c>
     </row>
     <row r="20">
@@ -585,7 +585,7 @@
         <v>0.09285714285714286</v>
       </c>
       <c r="G20" t="n">
-        <v>41.44978201739038</v>
+        <v>41.51474700445289</v>
       </c>
     </row>
     <row r="21">
@@ -593,7 +593,7 @@
         <v>0.1142857142857143</v>
       </c>
       <c r="G21" t="n">
-        <v>43.1235577771161</v>
+        <v>43.19114610267049</v>
       </c>
     </row>
     <row r="22">
@@ -601,7 +601,7 @@
         <v>0.1357142857142857</v>
       </c>
       <c r="G22" t="n">
-        <v>44.67573525963173</v>
+        <v>44.74575633844338</v>
       </c>
     </row>
     <row r="23">
@@ -609,7 +609,7 @@
         <v>0.1571428571428571</v>
       </c>
       <c r="G23" t="n">
-        <v>46.17833530939087</v>
+        <v>46.25071142618513</v>
       </c>
     </row>
     <row r="24">
@@ -617,7 +617,7 @@
         <v>0.1785714285714285</v>
       </c>
       <c r="G24" t="n">
-        <v>47.67249846719407</v>
+        <v>47.74721634683178</v>
       </c>
     </row>
     <row r="25">
@@ -625,7 +625,7 @@
         <v>0.2</v>
       </c>
       <c r="G25" t="n">
-        <v>49.18455741722726</v>
+        <v>49.26164491603944</v>
       </c>
     </row>
     <row r="26">
@@ -633,7 +633,7 @@
         <v>0.2214285714285714</v>
       </c>
       <c r="G26" t="n">
-        <v>50.73319712631989</v>
+        <v>50.81271096108785</v>
       </c>
     </row>
     <row r="27">
@@ -641,7 +641,7 @@
         <v>0.2428571428571429</v>
       </c>
       <c r="G27" t="n">
-        <v>52.33314787693456</v>
+        <v>52.4151667022551</v>
       </c>
     </row>
     <row r="28">
@@ -649,7 +649,7 @@
         <v>0.2642857142857143</v>
       </c>
       <c r="G28" t="n">
-        <v>53.99756867489796</v>
+        <v>54.08218893624242</v>
       </c>
     </row>
     <row r="29">
@@ -657,7 +657,7 @@
         <v>0.2857142857142857</v>
       </c>
       <c r="G29" t="n">
-        <v>55.7402498456779</v>
+        <v>55.82758313548739</v>
       </c>
     </row>
     <row r="30">
@@ -665,7 +665,7 @@
         <v>0.3071428571428571</v>
       </c>
       <c r="G30" t="n">
-        <v>57.57851574411401</v>
+        <v>57.66868698254237</v>
       </c>
     </row>
     <row r="31">
@@ -673,7 +673,7 @@
         <v>0.3285714285714286</v>
       </c>
       <c r="G31" t="n">
-        <v>59.53781456650842</v>
+        <v>59.63096062141042</v>
       </c>
     </row>
     <row r="32">
@@ -681,7 +681,7 @@
         <v>0.35</v>
       </c>
       <c r="G32" t="n">
-        <v>61.65930561667382</v>
+        <v>61.7555741318264</v>
       </c>
     </row>
     <row r="33">
@@ -689,7 +689,7 @@
         <v>0.3722413793103448</v>
       </c>
       <c r="G33" t="n">
-        <v>64.107382634362</v>
+        <v>64.20705854132522</v>
       </c>
     </row>
     <row r="34">
@@ -697,7 +697,7 @@
         <v>0.3944827586206897</v>
       </c>
       <c r="G34" t="n">
-        <v>66.93714549159543</v>
+        <v>67.04040776899865</v>
       </c>
     </row>
     <row r="35">
@@ -705,7 +705,7 @@
         <v>0.4167241379310345</v>
       </c>
       <c r="G35" t="n">
-        <v>70.37059327118469</v>
+        <v>70.47762898733734</v>
       </c>
     </row>
     <row r="36">
@@ -713,7 +713,7 @@
         <v>0.4389655172413793</v>
       </c>
       <c r="G36" t="n">
-        <v>74.76677174501124</v>
+        <v>74.8777744852522</v>
       </c>
     </row>
     <row r="37">
@@ -721,7 +721,7 @@
         <v>0.4612068965517241</v>
       </c>
       <c r="G37" t="n">
-        <v>80.6743348046122</v>
+        <v>80.78950293069431</v>
       </c>
     </row>
     <row r="38">
@@ -729,7 +729,7 @@
         <v>0.483448275862069</v>
       </c>
       <c r="G38" t="n">
-        <v>88.86390170202792</v>
+        <v>88.98343644210584</v>
       </c>
     </row>
     <row r="39">
@@ -737,7 +737,7 @@
         <v>0.5056896551724137</v>
       </c>
       <c r="G39" t="n">
-        <v>100.2814927661391</v>
+        <v>100.4055961494648</v>
       </c>
     </row>
     <row r="40">
@@ -745,7 +745,7 @@
         <v>0.5279310344827586</v>
       </c>
       <c r="G40" t="n">
-        <v>115.8338702170928</v>
+        <v>115.9627428807475</v>
       </c>
     </row>
     <row r="41">
@@ -753,7 +753,7 @@
         <v>0.5501724137931034</v>
       </c>
       <c r="G41" t="n">
-        <v>135.9539639016954</v>
+        <v>136.0878028077308</v>
       </c>
     </row>
     <row r="42">
@@ -761,7 +761,7 @@
         <v>0.5724137931034483</v>
       </c>
       <c r="G42" t="n">
-        <v>160.0870414419387</v>
+        <v>160.2260375520367</v>
       </c>
     </row>
     <row r="43">
@@ -769,7 +769,7 @@
         <v>0.5946551724137931</v>
       </c>
       <c r="G43" t="n">
-        <v>186.5044018843275</v>
+        <v>186.6487378452741</v>
       </c>
     </row>
     <row r="44">
@@ -777,7 +777,7 @@
         <v>0.6168965517241379</v>
       </c>
       <c r="G44" t="n">
-        <v>212.7929196452483</v>
+        <v>212.9427675419257</v>
       </c>
     </row>
     <row r="45">
@@ -785,7 +785,7 @@
         <v>0.6391379310344827</v>
       </c>
       <c r="G45" t="n">
-        <v>236.787582785058</v>
+        <v>236.9431020181425</v>
       </c>
     </row>
     <row r="46">
@@ -793,7 +793,7 @@
         <v>0.6613793103448276</v>
       </c>
       <c r="G46" t="n">
-        <v>257.2609323549592</v>
+        <v>257.4222676980625</v>
       </c>
     </row>
     <row r="47">
@@ -801,7 +801,7 @@
         <v>0.6836206896551724</v>
       </c>
       <c r="G47" t="n">
-        <v>273.9891394962529</v>
+        <v>274.156419382032</v>
       </c>
     </row>
     <row r="48">
@@ -809,7 +809,7 @@
         <v>0.7058620689655173</v>
       </c>
       <c r="G48" t="n">
-        <v>287.3987792885417</v>
+        <v>287.5721143656617</v>
       </c>
     </row>
     <row r="49">
@@ -817,7 +817,7 @@
         <v>0.728103448275862</v>
       </c>
       <c r="G49" t="n">
-        <v>298.1670906769376</v>
+        <v>298.3465726702042</v>
       </c>
     </row>
     <row r="50">
@@ -825,7 +825,7 @@
         <v>0.7503448275862069</v>
       </c>
       <c r="G50" t="n">
-        <v>306.9646750731542</v>
+        <v>307.1503759682462</v>
       </c>
     </row>
     <row r="51">
@@ -833,7 +833,7 @@
         <v>0.7725862068965517</v>
       </c>
       <c r="G51" t="n">
-        <v>314.3456723817574</v>
+        <v>314.5376439444732</v>
       </c>
     </row>
     <row r="52">
@@ -841,7 +841,7 @@
         <v>0.7948275862068965</v>
       </c>
       <c r="G52" t="n">
-        <v>320.7270477310917</v>
+        <v>320.9253213595649</v>
       </c>
     </row>
     <row r="53">
@@ -849,7 +849,7 @@
         <v>0.8170689655172414</v>
       </c>
       <c r="G53" t="n">
-        <v>326.4061475476524</v>
+        <v>326.6107344452251</v>
       </c>
     </row>
     <row r="54">
@@ -857,7 +857,7 @@
         <v>0.8393103448275863</v>
       </c>
       <c r="G54" t="n">
-        <v>331.5882161008475</v>
+        <v>331.7991077477811</v>
       </c>
     </row>
     <row r="55">
@@ -865,7 +865,7 @@
         <v>0.861551724137931</v>
       </c>
       <c r="G55" t="n">
-        <v>336.4119621606047</v>
+        <v>336.6291310549427</v>
       </c>
     </row>
     <row r="56">
@@ -873,7 +873,7 @@
         <v>0.8837931034482759</v>
       </c>
       <c r="G56" t="n">
-        <v>340.9697048139099</v>
+        <v>341.193105445876</v>
       </c>
     </row>
     <row r="57">
@@ -881,7 +881,7 @@
         <v>0.9060344827586206</v>
       </c>
       <c r="G57" t="n">
-        <v>345.3220873900977</v>
+        <v>345.5516574105022</v>
       </c>
     </row>
     <row r="58">
@@ -889,7 +889,7 @@
         <v>0.9282758620689655</v>
       </c>
       <c r="G58" t="n">
-        <v>349.5084111266541</v>
+        <v>349.7440726678673</v>
       </c>
     </row>
     <row r="59">
@@ -897,7 +897,7 @@
         <v>0.9505172413793104</v>
       </c>
       <c r="G59" t="n">
-        <v>353.5537431067759</v>
+        <v>353.7954042147502</v>
       </c>
     </row>
     <row r="60">
@@ -905,7 +905,7 @@
         <v>0.9727586206896551</v>
       </c>
       <c r="G60" t="n">
-        <v>357.4737524170749</v>
+        <v>357.7213085544115</v>
       </c>
     </row>
     <row r="61">
@@ -913,7 +913,7 @@
         <v>0.995</v>
       </c>
       <c r="G61" t="n">
-        <v>361.2779821816607</v>
+        <v>361.5313177645239</v>
       </c>
     </row>
     <row r="62">
@@ -938,7 +938,7 @@
         <v>0.995</v>
       </c>
       <c r="G63" t="n">
-        <v>361.2779821816607</v>
+        <v>362.2452190343664</v>
       </c>
     </row>
     <row r="64">
@@ -946,7 +946,7 @@
         <v>0.9727586206896551</v>
       </c>
       <c r="G64" t="n">
-        <v>358.7191453466932</v>
+        <v>361.5956896596138</v>
       </c>
     </row>
     <row r="65">
@@ -954,7 +954,7 @@
         <v>0.9505172413793104</v>
       </c>
       <c r="G65" t="n">
-        <v>355.8455007780256</v>
+        <v>360.7678175281587</v>
       </c>
     </row>
     <row r="66">
@@ -962,7 +962,7 @@
         <v>0.9282758620689655</v>
       </c>
       <c r="G66" t="n">
-        <v>352.8769603190232</v>
+        <v>359.7021361973303</v>
       </c>
     </row>
     <row r="67">
@@ -970,7 +970,7 @@
         <v>0.9060344827586206</v>
       </c>
       <c r="G67" t="n">
-        <v>349.7972796361406</v>
+        <v>358.3348661820444</v>
       </c>
     </row>
     <row r="68">
@@ -978,7 +978,7 @@
         <v>0.8837931034482759</v>
       </c>
       <c r="G68" t="n">
-        <v>346.5804016368072</v>
+        <v>356.595418537472</v>
       </c>
     </row>
     <row r="69">
@@ -986,7 +986,7 @@
         <v>0.861551724137931</v>
       </c>
       <c r="G69" t="n">
-        <v>343.233067805218</v>
+        <v>354.4022925828445</v>
       </c>
     </row>
     <row r="70">
@@ -994,7 +994,7 @@
         <v>0.8393103448275863</v>
       </c>
       <c r="G70" t="n">
-        <v>339.7371829699401</v>
+        <v>351.6566482774389</v>
       </c>
     </row>
     <row r="71">
@@ -1002,7 +1002,7 @@
         <v>0.8170689655172414</v>
       </c>
       <c r="G71" t="n">
-        <v>336.0696255387222</v>
+        <v>348.2325883316973</v>
       </c>
     </row>
     <row r="72">
@@ -1010,7 +1010,7 @@
         <v>0.7948275862068965</v>
       </c>
       <c r="G72" t="n">
-        <v>332.1583735761892</v>
+        <v>343.9629855947035</v>
       </c>
     </row>
     <row r="73">
@@ -1018,7 +1018,7 @@
         <v>0.7725862068965517</v>
       </c>
       <c r="G73" t="n">
-        <v>327.9445896621141</v>
+        <v>338.6197953601168</v>
       </c>
     </row>
     <row r="74">
@@ -1026,7 +1026,7 @@
         <v>0.7503448275862069</v>
       </c>
       <c r="G74" t="n">
-        <v>323.3670678475844</v>
+        <v>331.888856256828</v>
       </c>
     </row>
     <row r="75">
@@ -1034,7 +1034,7 @@
         <v>0.728103448275862</v>
       </c>
       <c r="G75" t="n">
-        <v>318.3145801471856</v>
+        <v>323.3426447556692</v>
       </c>
     </row>
     <row r="76">
@@ -1042,7 +1042,7 @@
         <v>0.7058620689655173</v>
       </c>
       <c r="G76" t="n">
-        <v>312.6326890582073</v>
+        <v>312.4228892839364</v>
       </c>
     </row>
     <row r="77">
@@ -1050,7 +1050,7 @@
         <v>0.6836206896551724</v>
       </c>
       <c r="G77" t="n">
-        <v>306.1073380258955</v>
+        <v>298.4613500820032</v>
       </c>
     </row>
     <row r="78">
@@ -1058,7 +1058,7 @@
         <v>0.6613793103448276</v>
       </c>
       <c r="G78" t="n">
-        <v>298.3924037847042</v>
+        <v>280.7896050953897</v>
       </c>
     </row>
     <row r="79">
@@ -1066,7 +1066,7 @@
         <v>0.6391379310344827</v>
       </c>
       <c r="G79" t="n">
-        <v>288.8726699865194</v>
+        <v>258.9962092426417</v>
       </c>
     </row>
     <row r="80">
@@ -1074,7 +1074,7 @@
         <v>0.6168965517241379</v>
       </c>
       <c r="G80" t="n">
-        <v>277.1550926364925</v>
+        <v>233.3261906049102</v>
       </c>
     </row>
     <row r="81">
@@ -1082,7 +1082,7 @@
         <v>0.5946551724137931</v>
       </c>
       <c r="G81" t="n">
-        <v>262.6646705647549</v>
+        <v>205.033934879284</v>
       </c>
     </row>
     <row r="82">
@@ -1090,7 +1090,7 @@
         <v>0.5724137931034483</v>
       </c>
       <c r="G82" t="n">
-        <v>244.9242752156728</v>
+        <v>176.3166742785506</v>
       </c>
     </row>
     <row r="83">
@@ -1098,7 +1098,7 @@
         <v>0.5501724137931034</v>
       </c>
       <c r="G83" t="n">
-        <v>223.8070970896839</v>
+        <v>149.6245288800276</v>
       </c>
     </row>
     <row r="84">
@@ -1106,7 +1106,7 @@
         <v>0.5279310344827586</v>
       </c>
       <c r="G84" t="n">
-        <v>199.8473261039421</v>
+        <v>126.7273721163916</v>
       </c>
     </row>
     <row r="85">
@@ -1114,7 +1114,7 @@
         <v>0.5056896551724137</v>
       </c>
       <c r="G85" t="n">
-        <v>174.424974095885</v>
+        <v>108.2246232750455</v>
       </c>
     </row>
     <row r="86">
@@ -1122,7 +1122,7 @@
         <v>0.483448275862069</v>
       </c>
       <c r="G86" t="n">
-        <v>149.5725493410216</v>
+        <v>93.73083366701991</v>
       </c>
     </row>
     <row r="87">
@@ -1130,7 +1130,7 @@
         <v>0.4612068965517241</v>
       </c>
       <c r="G87" t="n">
-        <v>127.3418132586263</v>
+        <v>82.38875127454155</v>
       </c>
     </row>
   </sheetData>
@@ -1174,7 +1174,7 @@
         <v>0.0004999999999999999</v>
       </c>
       <c r="C2" t="n">
-        <v>0.0002171356477331344</v>
+        <v>0.000216795859692289</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -1185,7 +1185,7 @@
         <v>0.0006667607160816619</v>
       </c>
       <c r="C3" t="n">
-        <v>0.0002212026169037217</v>
+        <v>0.000220856464603939</v>
       </c>
       <c r="D3" t="n">
         <v>1</v>
@@ -1196,7 +1196,7 @@
         <v>0.0008891397050194613</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0002266260074566472</v>
+        <v>0.0002262713682811721</v>
       </c>
       <c r="D4" t="n">
         <v>2</v>
@@ -1207,7 +1207,7 @@
         <v>0.001185686852830827</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0002338582149939655</v>
+        <v>0.0002334922583878623</v>
       </c>
       <c r="D5" t="n">
         <v>3</v>
@@ -1218,7 +1218,7 @@
         <v>0.001581138830084189</v>
       </c>
       <c r="C6" t="n">
-        <v>0.0002435025187468326</v>
+        <v>0.0002431214701044299</v>
       </c>
       <c r="D6" t="n">
         <v>4</v>
@@ -1229,7 +1229,7 @@
         <v>0.002108482517142911</v>
       </c>
       <c r="C7" t="n">
-        <v>0.000256363404499574</v>
+        <v>0.0002559622303033109</v>
       </c>
       <c r="D7" t="n">
         <v>5</v>
@@ -1240,7 +1240,7 @@
         <v>0.002811706625951745</v>
       </c>
       <c r="C8" t="n">
-        <v>0.0002735136712874585</v>
+        <v>0.0002730856592337885</v>
       </c>
       <c r="D8" t="n">
         <v>6</v>
@@ -1251,7 +1251,7 @@
         <v>0.003749471046662279</v>
       </c>
       <c r="C9" t="n">
-        <v>0.0002963839196164216</v>
+        <v>0.0002959201187047061</v>
       </c>
       <c r="D9" t="n">
         <v>7</v>
@@ -1262,7 +1262,7 @@
         <v>0.004999999999999999</v>
       </c>
       <c r="C10" t="n">
-        <v>0.0003268818859219913</v>
+        <v>0.0003263703598010394</v>
       </c>
       <c r="D10" t="n">
         <v>8</v>
@@ -1273,7 +1273,7 @@
         <v>0.006667607160816619</v>
       </c>
       <c r="C11" t="n">
-        <v>0.0003675515776278646</v>
+        <v>0.0003669764089175414</v>
       </c>
       <c r="D11" t="n">
         <v>9</v>
@@ -1284,7 +1284,7 @@
         <v>0.008891397050194613</v>
       </c>
       <c r="C12" t="n">
-        <v>0.0004217854831571319</v>
+        <v>0.0004211254456898839</v>
       </c>
       <c r="D12" t="n">
         <v>10</v>
@@ -1295,7 +1295,7 @@
         <v>0.01185686852830828</v>
       </c>
       <c r="C13" t="n">
-        <v>0.0004941075585304203</v>
+        <v>0.0004933343467568917</v>
       </c>
       <c r="D13" t="n">
         <v>11</v>
@@ -1306,7 +1306,7 @@
         <v>0.0158113883008419</v>
       </c>
       <c r="C14" t="n">
-        <v>0.0005905505960600264</v>
+        <v>0.0005896264639235013</v>
       </c>
       <c r="D14" t="n">
         <v>12</v>
@@ -1317,7 +1317,7 @@
         <v>0.02108482517142911</v>
       </c>
       <c r="C15" t="n">
-        <v>0.0007191594535958868</v>
+        <v>0.0007180340659207448</v>
       </c>
       <c r="D15" t="n">
         <v>13</v>
@@ -1328,7 +1328,7 @@
         <v>0.02811706625951745</v>
       </c>
       <c r="C16" t="n">
-        <v>0.0008906621215521796</v>
+        <v>0.0008892683553028463</v>
       </c>
       <c r="D16" t="n">
         <v>14</v>
@@ -1339,7 +1339,7 @@
         <v>0.03749471046662279</v>
       </c>
       <c r="C17" t="n">
-        <v>0.001119364605561117</v>
+        <v>0.001117612950730202</v>
       </c>
       <c r="D17" t="n">
         <v>15</v>
@@ -1350,7 +1350,7 @@
         <v>0.05</v>
       </c>
       <c r="C18" t="n">
-        <v>0.001424344275362326</v>
+        <v>0.001422115368428492</v>
       </c>
       <c r="D18" t="n">
         <v>16</v>
@@ -1361,7 +1361,7 @@
         <v>0.07142857142857142</v>
       </c>
       <c r="C19" t="n">
-        <v>0.00194694552387337</v>
+        <v>0.00194389881637929</v>
       </c>
       <c r="D19" t="n">
         <v>17</v>
@@ -1372,7 +1372,7 @@
         <v>0.09285714285714286</v>
       </c>
       <c r="C20" t="n">
-        <v>0.002469547479923129</v>
+        <v>0.002465682970762896</v>
       </c>
       <c r="D20" t="n">
         <v>18</v>
@@ -1383,7 +1383,7 @@
         <v>0.1142857142857143</v>
       </c>
       <c r="C21" t="n">
-        <v>0.002992152427019559</v>
+        <v>0.002987470111531449</v>
       </c>
       <c r="D21" t="n">
         <v>19</v>
@@ -1394,7 +1394,7 @@
         <v>0.1357142857142857</v>
       </c>
       <c r="C22" t="n">
-        <v>0.003514766852204777</v>
+        <v>0.003509266715724765</v>
       </c>
       <c r="D22" t="n">
         <v>20</v>
@@ -1405,7 +1405,7 @@
         <v>0.1571428571428571</v>
       </c>
       <c r="C23" t="n">
-        <v>0.004037405781671539</v>
+        <v>0.004031087786912336</v>
       </c>
       <c r="D23" t="n">
         <v>21</v>
@@ -1416,7 +1416,7 @@
         <v>0.1785714285714285</v>
       </c>
       <c r="C24" t="n">
-        <v>0.004560098827155541</v>
+        <v>0.004552962894605495</v>
       </c>
       <c r="D24" t="n">
         <v>22</v>
@@ -1427,7 +1427,7 @@
         <v>0.2</v>
       </c>
       <c r="C25" t="n">
-        <v>0.00508289620010763</v>
+        <v>0.005074942187295917</v>
       </c>
       <c r="D25" t="n">
         <v>23</v>
@@ -1438,7 +1438,7 @@
         <v>0.2214285714285714</v>
       </c>
       <c r="C26" t="n">
-        <v>0.005605869250002869</v>
+        <v>0.005597096953606071</v>
       </c>
       <c r="D26" t="n">
         <v>24</v>
@@ -1449,7 +1449,7 @@
         <v>0.2428571428571429</v>
       </c>
       <c r="C27" t="n">
-        <v>0.006129092745107013</v>
+        <v>0.006119501990772683</v>
       </c>
       <c r="D27" t="n">
         <v>25</v>
@@ -1460,7 +1460,7 @@
         <v>0.2642857142857143</v>
       </c>
       <c r="C28" t="n">
-        <v>0.006652582880789357</v>
+        <v>0.006642173847555667</v>
       </c>
       <c r="D28" t="n">
         <v>26</v>
@@ -1471,7 +1471,7 @@
         <v>0.2857142857142857</v>
       </c>
       <c r="C29" t="n">
-        <v>0.007176142932753934</v>
+        <v>0.00716491700937947</v>
       </c>
       <c r="D29" t="n">
         <v>27</v>
@@ -1482,7 +1482,7 @@
         <v>0.3071428571428571</v>
       </c>
       <c r="C30" t="n">
-        <v>0.007699034324577588</v>
+        <v>0.007686996050497242</v>
       </c>
       <c r="D30" t="n">
         <v>28</v>
@@ -1493,7 +1493,7 @@
         <v>0.3285714285714286</v>
       </c>
       <c r="C31" t="n">
-        <v>0.00821934271001842</v>
+        <v>0.008206503752883612</v>
       </c>
       <c r="D31" t="n">
         <v>29</v>
@@ -1504,7 +1504,7 @@
         <v>0.35</v>
       </c>
       <c r="C32" t="n">
-        <v>0.00873285115808908</v>
+        <v>0.00871923783450078</v>
       </c>
       <c r="D32" t="n">
         <v>30</v>
@@ -1515,7 +1515,7 @@
         <v>0.3722413793103448</v>
       </c>
       <c r="C33" t="n">
-        <v>0.009249620561678298</v>
+        <v>0.009235261325489996</v>
       </c>
       <c r="D33" t="n">
         <v>31</v>
@@ -1526,7 +1526,7 @@
         <v>0.3944827586206897</v>
       </c>
       <c r="C34" t="n">
-        <v>0.009732722138487533</v>
+        <v>0.009717730835677802</v>
       </c>
       <c r="D34" t="n">
         <v>32</v>
@@ -1537,7 +1537,7 @@
         <v>0.4167241379310345</v>
       </c>
       <c r="C35" t="n">
-        <v>0.01015274410602545</v>
+        <v>0.01013732494037079</v>
       </c>
       <c r="D35" t="n">
         <v>33</v>
@@ -1548,7 +1548,7 @@
         <v>0.4389655172413793</v>
       </c>
       <c r="C36" t="n">
-        <v>0.01046483105595749</v>
+        <v>0.01044931744151909</v>
       </c>
       <c r="D36" t="n">
         <v>34</v>
@@ -1559,7 +1559,7 @@
         <v>0.4612068965517241</v>
       </c>
       <c r="C37" t="n">
-        <v>0.01061056161260175</v>
+        <v>0.01059543590377482</v>
       </c>
       <c r="D37" t="n">
         <v>35</v>
@@ -1570,7 +1570,7 @@
         <v>0.483448275862069</v>
       </c>
       <c r="C38" t="n">
-        <v>0.01053199932493651</v>
+        <v>0.01051785130085311</v>
       </c>
       <c r="D38" t="n">
         <v>36</v>
@@ -1652,7 +1652,7 @@
         <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>2.032677093376522e-07</v>
+        <v>2.035363096056934e-07</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
@@ -1663,828 +1663,828 @@
     </row>
     <row r="3">
       <c r="C3" t="n">
-        <v>1.081180751076608</v>
+        <v>1.056072900399631</v>
       </c>
       <c r="D3" t="n">
-        <v>6.209920818022901e-07</v>
+        <v>4.466085586143215e-07</v>
       </c>
       <c r="E3" t="n">
-        <v>3.34570144634943e-08</v>
+        <v>1.822775422051591e-08</v>
       </c>
       <c r="F3" t="n">
-        <v>6.430390910772506e-05</v>
+        <v>3.546129948402715e-05</v>
       </c>
     </row>
     <row r="4">
       <c r="C4" t="n">
-        <v>1.168951816498578</v>
+        <v>1.115289970958488</v>
       </c>
       <c r="D4" t="n">
-        <v>1.80511400802517e-06</v>
+        <v>9.564444534568073e-07</v>
       </c>
       <c r="E4" t="n">
-        <v>1.399279726289374e-07</v>
+        <v>5.977009882733255e-08</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0002535744608960218</v>
+        <v>0.0001119889865966528</v>
       </c>
     </row>
     <row r="5">
       <c r="C5" t="n">
-        <v>1.263848202934298</v>
+        <v>1.17782751441675</v>
       </c>
       <c r="D5" t="n">
-        <v>4.992569446659943e-06</v>
+        <v>1.999125369282718e-06</v>
       </c>
       <c r="E5" t="n">
-        <v>4.624657706206858e-07</v>
+        <v>1.521871369440833e-07</v>
       </c>
       <c r="F5" t="n">
-        <v>0.000783889810148505</v>
+        <v>0.0002731966677663386</v>
       </c>
     </row>
     <row r="6">
       <c r="C6" t="n">
-        <v>1.366448349295325</v>
+        <v>1.243871719320585</v>
       </c>
       <c r="D6" t="n">
-        <v>1.313846102722152e-05</v>
+        <v>4.07819393047704e-06</v>
       </c>
       <c r="E6" t="n">
-        <v>1.39258896076893e-06</v>
+        <v>3.528729974937648e-07</v>
       </c>
       <c r="F6" t="n">
-        <v>0.002198366347951525</v>
+        <v>0.0006046760814835724</v>
       </c>
     </row>
     <row r="7">
       <c r="C7" t="n">
-        <v>1.477377652598511</v>
+        <v>1.313619214347965</v>
       </c>
       <c r="D7" t="n">
-        <v>3.289771879566346e-05</v>
+        <v>8.119761694627957e-06</v>
       </c>
       <c r="E7" t="n">
-        <v>3.945969638015334e-06</v>
+        <v>7.782614221468724e-07</v>
       </c>
       <c r="F7" t="n">
-        <v>0.005789838787609912</v>
+        <v>0.001269997579289105</v>
       </c>
     </row>
     <row r="8">
       <c r="C8" t="n">
-        <v>1.597312280060254</v>
+        <v>1.387277653717139</v>
       </c>
       <c r="D8" t="n">
-        <v>7.837688071378681e-05</v>
+        <v>1.577851978814465e-05</v>
       </c>
       <c r="E8" t="n">
-        <v>1.061880845707563e-05</v>
+        <v>1.658416480960007e-06</v>
       </c>
       <c r="F8" t="n">
-        <v>0.0144708296715136</v>
+        <v>0.002573498011637963</v>
       </c>
     </row>
     <row r="9">
       <c r="C9" t="n">
-        <v>1.726983290659435</v>
+        <v>1.465066335420654</v>
       </c>
       <c r="D9" t="n">
-        <v>0.0001776687597655306</v>
+        <v>2.992518198801463e-05</v>
       </c>
       <c r="E9" t="n">
-        <v>2.721965693730942e-05</v>
+        <v>3.436031836029004e-06</v>
       </c>
       <c r="F9" t="n">
-        <v>0.03444600712138134</v>
+        <v>0.005066346506543844</v>
       </c>
     </row>
     <row r="10">
       <c r="C10" t="n">
-        <v>1.86718109129192</v>
+        <v>1.547216854125548</v>
       </c>
       <c r="D10" t="n">
-        <v>0.0003832084443382996</v>
+        <v>5.539300268903446e-05</v>
       </c>
       <c r="E10" t="n">
-        <v>6.653653215743658e-05</v>
+        <v>6.94049839911876e-06</v>
       </c>
       <c r="F10" t="n">
-        <v>0.07820235328914468</v>
+        <v>0.009719915035892776</v>
       </c>
     </row>
     <row r="11">
       <c r="C11" t="n">
-        <v>2.018760254679039</v>
+        <v>1.633973790683559</v>
       </c>
       <c r="D11" t="n">
-        <v>0.0007864298235623324</v>
+        <v>0.0001000738437390725</v>
       </c>
       <c r="E11" t="n">
-        <v>0.0001551829272144047</v>
+        <v>1.368441206533745e-05</v>
       </c>
       <c r="F11" t="n">
-        <v>0.1694506631987927</v>
+        <v>0.01819965035414293</v>
       </c>
     </row>
     <row r="12">
       <c r="C12" t="n">
-        <v>2.182644728397487</v>
+        <v>1.725595440304165</v>
       </c>
       <c r="D12" t="n">
-        <v>0.001535627155017469</v>
+        <v>0.0001764549395764542</v>
       </c>
       <c r="E12" t="n">
-        <v>0.0003454574701538053</v>
+        <v>2.635242371281127e-05</v>
       </c>
       <c r="F12" t="n">
-        <v>0.3506039142715516</v>
+        <v>0.03328255030527671</v>
       </c>
     </row>
     <row r="13">
       <c r="C13" t="n">
-        <v>2.359833466782194</v>
+        <v>1.822354581558397</v>
       </c>
       <c r="D13" t="n">
-        <v>0.002853070452997091</v>
+        <v>0.0003036649209266178</v>
       </c>
       <c r="E13" t="n">
-        <v>0.0007342713663118464</v>
+        <v>4.95804164135007e-05</v>
       </c>
       <c r="F13" t="n">
-        <v>0.6929843325821001</v>
+        <v>0.05947005864959715</v>
       </c>
     </row>
     <row r="14">
       <c r="C14" t="n">
-        <v>2.551406520031289</v>
+        <v>1.924539288502931</v>
       </c>
       <c r="D14" t="n">
-        <v>0.005043593929536577</v>
+        <v>0.0005100385434217211</v>
       </c>
       <c r="E14" t="n">
-        <v>0.001490665419434521</v>
+        <v>9.115444143559446e-05</v>
       </c>
       <c r="F14" t="n">
-        <v>1.309035720951284</v>
+        <v>0.1038524473308258</v>
       </c>
     </row>
     <row r="15">
       <c r="C15" t="n">
-        <v>2.758531617629183</v>
+        <v>2.032453788342332</v>
       </c>
       <c r="D15" t="n">
-        <v>0.008483374410772631</v>
+        <v>0.0008361013680726838</v>
       </c>
       <c r="E15" t="n">
-        <v>0.002891552738279606</v>
+        <v>0.0001637884490669811</v>
       </c>
       <c r="F15" t="n">
-        <v>2.364330364713223</v>
+        <v>0.1772758839867167</v>
       </c>
     </row>
     <row r="16">
       <c r="C16" t="n">
-        <v>2.982471286216891</v>
+        <v>2.146419367182903</v>
       </c>
       <c r="D16" t="n">
-        <v>0.01357682001579758</v>
+        <v>0.001337711428066221</v>
       </c>
       <c r="E16" t="n">
-        <v>0.005361629052712869</v>
+        <v>0.0002876583658684868</v>
       </c>
       <c r="F16" t="n">
-        <v>4.085337203276906</v>
+        <v>0.2958436530396987</v>
       </c>
     </row>
     <row r="17">
       <c r="C17" t="n">
-        <v>3.224590545296395</v>
+        <v>2.266775326574788</v>
       </c>
       <c r="D17" t="n">
-        <v>0.02067418465386701</v>
+        <v>0.002088880070657771</v>
       </c>
       <c r="E17" t="n">
-        <v>0.009508042989386786</v>
+        <v>0.0004938637195049883</v>
       </c>
       <c r="F17" t="n">
-        <v>6.75739947636241</v>
+        <v>0.4827425940070409</v>
       </c>
     </row>
     <row r="18">
       <c r="C18" t="n">
-        <v>3.486365227678085</v>
+        <v>2.393879993690156</v>
       </c>
       <c r="D18" t="n">
-        <v>0.02995433106391986</v>
+        <v>0.003183553419202047</v>
       </c>
       <c r="E18" t="n">
-        <v>0.01613467480012682</v>
+        <v>0.0008289391713132632</v>
       </c>
       <c r="F18" t="n">
-        <v>10.70713899777364</v>
+        <v>0.7703205664448112</v>
       </c>
     </row>
     <row r="19">
       <c r="C19" t="n">
-        <v>3.769390975388362</v>
+        <v>2.528111788145012</v>
       </c>
       <c r="D19" t="n">
-        <v>0.04129445743151074</v>
+        <v>0.004735418241109286</v>
       </c>
       <c r="E19" t="n">
-        <v>0.02621729561881212</v>
+        <v>0.001360428059413633</v>
       </c>
       <c r="F19" t="n">
-        <v>16.26555112547118</v>
+        <v>1.202250493724945</v>
       </c>
     </row>
     <row r="20">
       <c r="C20" t="n">
-        <v>4.075392965871777</v>
+        <v>2.669870348640799</v>
       </c>
       <c r="D20" t="n">
-        <v>0.0541657558045136</v>
+        <v>0.006874674020479963</v>
       </c>
       <c r="E20" t="n">
-        <v>0.04082280324990949</v>
+        <v>0.002183343042526717</v>
       </c>
       <c r="F20" t="n">
-        <v>23.7127964494775</v>
+        <v>1.835507755068237</v>
       </c>
     </row>
     <row r="21">
       <c r="C21" t="n">
-        <v>4.406236427773572</v>
+        <v>2.819577722780061</v>
       </c>
       <c r="D21" t="n">
-        <v>0.06760187707523639</v>
+        <v>0.009740773455670594</v>
       </c>
       <c r="E21" t="n">
-        <v>0.06096581585467114</v>
+        <v>0.003427070548428385</v>
       </c>
       <c r="F21" t="n">
-        <v>33.21239218510505</v>
+        <v>2.741775554468149</v>
       </c>
     </row>
     <row r="22">
       <c r="C22" t="n">
-        <v>4.763938010401341</v>
+        <v>2.977679623598525</v>
       </c>
       <c r="D22" t="n">
-        <v>0.08027745704450175</v>
+        <v>0.0134704573753935</v>
       </c>
       <c r="E22" t="n">
-        <v>0.0874141517809566</v>
+        <v>0.005261940405792061</v>
       </c>
       <c r="F22" t="n">
-        <v>44.74906953169185</v>
+        <v>4.007801709756823</v>
       </c>
     </row>
     <row r="23">
       <c r="C23" t="n">
-        <v>5.150678076168123</v>
+        <v>3.144646756554574</v>
       </c>
       <c r="D23" t="n">
-        <v>0.09070461056359774</v>
+        <v>0.01818104354655484</v>
       </c>
       <c r="E23" t="n">
-        <v>0.120476959816805</v>
+        <v>0.007904320587138795</v>
       </c>
       <c r="F23" t="n">
-        <v>58.08808649297832</v>
+        <v>5.734191331788478</v>
       </c>
     </row>
     <row r="24">
       <c r="C24" t="n">
-        <v>5.56881399094527</v>
+        <v>3.320976220926879</v>
       </c>
       <c r="D24" t="n">
-        <v>0.09751378716587029</v>
+        <v>0.02394985222187419</v>
       </c>
       <c r="E24" t="n">
-        <v>0.159827395773055</v>
+        <v>0.01161877972932506</v>
       </c>
       <c r="F24" t="n">
-        <v>72.77178072396683</v>
+        <v>8.032165807023437</v>
       </c>
     </row>
     <row r="25">
       <c r="C25" t="n">
-        <v>6.02089449333613</v>
+        <v>3.507192989792454</v>
       </c>
       <c r="D25" t="n">
-        <v>0.09974786031094586</v>
+        <v>0.03079175446418437</v>
       </c>
       <c r="E25" t="n">
-        <v>0.2044164681199389</v>
+        <v>0.01671568228911904</v>
       </c>
       <c r="F25" t="n">
-        <v>88.16097620109484</v>
+        <v>11.01797497636418</v>
       </c>
     </row>
     <row r="26">
       <c r="C26" t="n">
-        <v>6.50967523045817</v>
+        <v>3.703851472991369</v>
       </c>
       <c r="D26" t="n">
-        <v>0.09708274727152098</v>
+        <v>0.038637907456604</v>
       </c>
       <c r="E26" t="n">
-        <v>0.2525199728511075</v>
+        <v>0.02354264829029689</v>
       </c>
       <c r="F26" t="n">
-        <v>103.5165444765979</v>
+        <v>14.80492486214663</v>
       </c>
     </row>
     <row r="27">
       <c r="C27" t="n">
-        <v>7.038135554931555</v>
+        <v>3.911537167731438</v>
       </c>
       <c r="D27" t="n">
-        <v>0.08990450021945515</v>
+        <v>0.04731951959683757</v>
       </c>
       <c r="E27" t="n">
-        <v>0.3019276435918406</v>
+        <v>0.0324687122681283</v>
       </c>
       <c r="F27" t="n">
-        <v>118.1041915949103</v>
+        <v>19.49336002885624</v>
       </c>
     </row>
     <row r="28">
       <c r="C28" t="n">
-        <v>7.609496685459877</v>
+        <v>4.130868401747096</v>
       </c>
       <c r="D28" t="n">
-        <v>0.07921760514926471</v>
+        <v>0.05656067995554884</v>
       </c>
       <c r="E28" t="n">
-        <v>0.3502425422522416</v>
+        <v>0.04386079844693717</v>
       </c>
       <c r="F28" t="n">
-        <v>131.2981052233999</v>
+        <v>25.15936932440463</v>
       </c>
     </row>
     <row r="29">
       <c r="C29" t="n">
-        <v>8.22724134170047</v>
+        <v>4.362498174202242</v>
       </c>
       <c r="D29" t="n">
-        <v>0.06641449751535451</v>
+        <v>0.06598367233797323</v>
       </c>
       <c r="E29" t="n">
-        <v>0.3952242688513165</v>
+        <v>0.058053258665643</v>
       </c>
       <c r="F29" t="n">
-        <v>142.6594667669021</v>
+        <v>31.84339036213758</v>
       </c>
     </row>
     <row r="30">
       <c r="C30" t="n">
-        <v>8.895134973108235</v>
+        <v>4.607116099817854</v>
       </c>
       <c r="D30" t="n">
-        <v>0.0529791489650123</v>
+        <v>0.07512870613571553</v>
       </c>
       <c r="E30" t="n">
-        <v>0.43509539690871</v>
+        <v>0.07531256731610247</v>
       </c>
       <c r="F30" t="n">
-        <v>151.9738580229593</v>
+        <v>39.54018004481098</v>
       </c>
     </row>
     <row r="31">
       <c r="C31" t="n">
-        <v>9.617248711152964</v>
+        <v>4.865450462012474</v>
       </c>
       <c r="D31" t="n">
-        <v>0.04021128655721818</v>
+        <v>0.08348777794557297</v>
       </c>
       <c r="E31" t="n">
-        <v>0.4687424437811971</v>
+        <v>0.09580061144044882</v>
       </c>
       <c r="F31" t="n">
-        <v>159.2440286171639</v>
+        <v>48.19170821961541</v>
       </c>
     </row>
     <row r="32">
       <c r="C32" t="n">
-        <v>10.3979841848149</v>
+        <v>5.138270381168236</v>
       </c>
       <c r="D32" t="n">
-        <v>0.02903968249718157</v>
+        <v>0.09054979284858396</v>
       </c>
       <c r="E32" t="n">
-        <v>0.4957757878443145</v>
+        <v>0.1195410694375124</v>
       </c>
       <c r="F32" t="n">
-        <v>164.6465826026463</v>
+        <v>57.68435935181763</v>
       </c>
     </row>
     <row r="33">
       <c r="C33" t="n">
-        <v>11.24210035062087</v>
+        <v>5.426388104477853</v>
       </c>
       <c r="D33" t="n">
-        <v>0.0199543076264745</v>
+        <v>0.09585164836966344</v>
       </c>
       <c r="E33" t="n">
-        <v>0.5164540973896725</v>
+        <v>0.1463938488702289</v>
       </c>
       <c r="F33" t="n">
-        <v>168.4688060346291</v>
+        <v>67.85138158701835</v>
       </c>
     </row>
     <row r="34">
       <c r="C34" t="n">
-        <v>12.15474250076286</v>
+        <v>5.73066142418998</v>
       </c>
       <c r="D34" t="n">
-        <v>0.01304614998585794</v>
+        <v>0.09902828927375873</v>
       </c>
       <c r="E34" t="n">
-        <v>0.531512901685167</v>
+        <v>0.1760422316562571</v>
       </c>
       <c r="F34" t="n">
-        <v>171.0433079691248</v>
+        <v>78.48085229425048</v>
       </c>
     </row>
     <row r="35">
       <c r="C35" t="n">
-        <v>13.14147362611756</v>
+        <v>6.05199623145259</v>
       </c>
       <c r="D35" t="n">
-        <v>0.008115755883959318</v>
+        <v>0.0998542452363739</v>
       </c>
       <c r="E35" t="n">
-        <v>0.5419534572819544</v>
+        <v>0.2079961721036135</v>
       </c>
       <c r="F35" t="n">
-        <v>172.6942356089615</v>
+        <v>89.32863940009211</v>
       </c>
     </row>
     <row r="36">
       <c r="C36" t="n">
-        <v>14.20830832533922</v>
+        <v>6.39134921335777</v>
       </c>
       <c r="D36" t="n">
-        <v>0.004803706755312397</v>
+        <v>0.09827009050458772</v>
       </c>
       <c r="E36" t="n">
-        <v>0.5488449228013909</v>
+        <v>0.2416132141644526</v>
       </c>
       <c r="F36" t="n">
-        <v>173.7021362250129</v>
+        <v>100.1350715480831</v>
       </c>
     </row>
     <row r="37">
       <c r="C37" t="n">
-        <v>15.36174946671828</v>
+        <v>6.749730701217637</v>
       </c>
       <c r="D37" t="n">
-        <v>0.002705359004407944</v>
+        <v>0.09438951285343933</v>
       </c>
       <c r="E37" t="n">
-        <v>0.553175555491682</v>
+        <v>0.2761360318154235</v>
       </c>
       <c r="F37" t="n">
-        <v>174.2879494446887</v>
+        <v>110.6434370326214</v>
       </c>
     </row>
     <row r="38">
       <c r="C38" t="n">
-        <v>16.60882782627716</v>
+        <v>7.128207678551341</v>
       </c>
       <c r="D38" t="n">
-        <v>0.001449686938066563</v>
+        <v>0.08848582396664992</v>
       </c>
       <c r="E38" t="n">
-        <v>0.5557663894305984</v>
+        <v>0.3107430841696986</v>
       </c>
       <c r="F38" t="n">
-        <v>174.6121017319837</v>
+        <v>120.6181325262186</v>
       </c>
     </row>
     <row r="39">
       <c r="C39" t="n">
-        <v>17.9571449437164</v>
+        <v>7.527906957738633</v>
       </c>
       <c r="D39" t="n">
-        <v>0.0007391361634621528</v>
+        <v>0.08096013430326376</v>
       </c>
       <c r="E39" t="n">
-        <v>0.5572420032580172</v>
+        <v>0.3446067978605409</v>
       </c>
       <c r="F39" t="n">
-        <v>174.7828608582768</v>
+        <v>129.8603401729826</v>
       </c>
     </row>
     <row r="40">
       <c r="C40" t="n">
-        <v>19.41491945743881</v>
+        <v>7.950018534797596</v>
       </c>
       <c r="D40" t="n">
-        <v>0.0003585713458110124</v>
+        <v>0.0722963391373603</v>
       </c>
       <c r="E40" t="n">
-        <v>0.5580421082732873</v>
+        <v>0.3769524637097993</v>
       </c>
       <c r="F40" t="n">
-        <v>174.8684975527534</v>
+        <v>138.219513594474</v>
       </c>
     </row>
     <row r="41">
       <c r="C41" t="n">
-        <v>20.99103720108555</v>
+        <v>8.395799132274519</v>
       </c>
       <c r="D41" t="n">
-        <v>0.0001655112868827408</v>
+        <v>0.06300992447815119</v>
       </c>
       <c r="E41" t="n">
-        <v>0.5584551162415501</v>
+        <v>0.4071109172282457</v>
       </c>
       <c r="F41" t="n">
-        <v>174.909383402506</v>
+        <v>145.5996163541418</v>
       </c>
     </row>
     <row r="42">
       <c r="C42" t="n">
-        <v>22.69510536694668</v>
+        <v>8.866575940793851</v>
       </c>
       <c r="D42" t="n">
-        <v>7.269098502103429e-05</v>
+        <v>0.05359807321448942</v>
       </c>
       <c r="E42" t="n">
-        <v>0.5586580726958436</v>
+        <v>0.4345590877290312</v>
       </c>
       <c r="F42" t="n">
-        <v>174.9279665451103</v>
+        <v>151.9598467128503</v>
       </c>
     </row>
     <row r="43">
       <c r="C43" t="n">
-        <v>24.53751106639818</v>
+        <v>9.363750570407745</v>
       </c>
       <c r="D43" t="n">
-        <v>3.03762666710017e-05</v>
+        <v>0.0444976383604419</v>
       </c>
       <c r="E43" t="n">
-        <v>0.5587530185418157</v>
+        <v>0.4589444372635201</v>
       </c>
       <c r="F43" t="n">
-        <v>174.9360072469085</v>
+        <v>157.3103486952488</v>
       </c>
     </row>
     <row r="44">
       <c r="C44" t="n">
-        <v>26.52948464431896</v>
+        <v>9.888803223509203</v>
       </c>
       <c r="D44" t="n">
-        <v>1.207783643852829e-05</v>
+        <v>0.03605556559316728</v>
       </c>
       <c r="E44" t="n">
-        <v>0.55879530226765</v>
+        <v>0.4800917739893528</v>
       </c>
       <c r="F44" t="n">
-        <v>174.9393192667558</v>
+        <v>161.7040175980236</v>
       </c>
     </row>
     <row r="45">
       <c r="C45" t="n">
-        <v>28.6831681334201</v>
+        <v>10.44329710173258</v>
       </c>
       <c r="D45" t="n">
-        <v>4.569248684690873e-06</v>
+        <v>0.02851380853410374</v>
       </c>
       <c r="E45" t="n">
-        <v>0.5588132285438357</v>
+        <v>0.4979934353264962</v>
       </c>
       <c r="F45" t="n">
-        <v>174.9406179745906</v>
+        <v>165.2258694580439</v>
       </c>
     </row>
     <row r="46">
       <c r="C46" t="n">
-        <v>31.01168926574779</v>
+        <v>11.02888305996178</v>
       </c>
       <c r="D46" t="n">
-        <v>1.644755515183486e-06</v>
+        <v>0.0220082601736352</v>
       </c>
       <c r="E46" t="n">
-        <v>0.5588204632638837</v>
+        <v>0.5127859423344675</v>
       </c>
       <c r="F46" t="n">
-        <v>174.9411027547116</v>
+        <v>167.9815294602566</v>
       </c>
     </row>
     <row r="47">
       <c r="C47" t="n">
-        <v>33.52924149249557</v>
+        <v>11.64730452130219</v>
       </c>
       <c r="D47" t="n">
-        <v>5.633247226257583e-07</v>
+        <v>0.01657920722567885</v>
       </c>
       <c r="E47" t="n">
-        <v>0.5588232427425435</v>
+        <v>0.5247176013237221</v>
       </c>
       <c r="F47" t="n">
-        <v>174.9412750161666</v>
+        <v>170.0862322806043</v>
       </c>
     </row>
     <row r="48">
       <c r="C48" t="n">
-        <v>36.25117049988533</v>
+        <v>12.30040266764933</v>
       </c>
       <c r="D48" t="n">
-        <v>1.835765382727007e-07</v>
+        <v>0.01218959774672811</v>
       </c>
       <c r="E48" t="n">
-        <v>0.5588242592486473</v>
+        <v>0.5341120279237729</v>
       </c>
       <c r="F48" t="n">
-        <v>174.9413332850174</v>
+        <v>171.6553890313407</v>
       </c>
     </row>
     <row r="49">
       <c r="C49" t="n">
-        <v>39.19406774847219</v>
+        <v>12.99012192130778</v>
       </c>
       <c r="D49" t="n">
-        <v>5.692151425673902e-08</v>
+        <v>0.008747069044319744</v>
       </c>
       <c r="E49" t="n">
-        <v>0.5588246131291759</v>
+        <v>0.5413322390203815</v>
       </c>
       <c r="F49" t="n">
-        <v>174.9413520472633</v>
+        <v>172.797352073066</v>
       </c>
     </row>
     <row r="50">
       <c r="C50" t="n">
-        <v>42.37587160604063</v>
+        <v>13.71851573398033</v>
       </c>
       <c r="D50" t="n">
-        <v>1.679332210582987e-08</v>
+        <v>0.006126088985510457</v>
       </c>
       <c r="E50" t="n">
-        <v>0.5588247304022512</v>
+        <v>0.5467489971622962</v>
       </c>
       <c r="F50" t="n">
-        <v>174.941357798062</v>
+        <v>173.608588978793</v>
       </c>
     </row>
     <row r="51">
       <c r="C51" t="n">
-        <v>45.81597669054491</v>
+        <v>14.48775270036257</v>
       </c>
       <c r="D51" t="n">
-        <v>4.714088110396602e-09</v>
+        <v>0.00418746907975341</v>
       </c>
       <c r="E51" t="n">
-        <v>0.5588247673961269</v>
+        <v>0.5507157822216615</v>
       </c>
       <c r="F51" t="n">
-        <v>174.9413594759439</v>
+        <v>174.1711284821802</v>
       </c>
     </row>
     <row r="52">
       <c r="C52" t="n">
-        <v>49.5353520895917</v>
+        <v>15.30012301454448</v>
       </c>
       <c r="D52" t="n">
-        <v>1.259098415669535e-09</v>
+        <v>0.002793621030976338</v>
       </c>
       <c r="E52" t="n">
-        <v>0.5588247785043884</v>
+        <v>0.5535513974049544</v>
       </c>
       <c r="F52" t="n">
-        <v>174.9413599419368</v>
+        <v>174.55190288992</v>
       </c>
     </row>
     <row r="53">
       <c r="C53" t="n">
-        <v>53.55666917706899</v>
+        <v>16.15804528844113</v>
       </c>
       <c r="D53" t="n">
-        <v>3.199798007556998e-10</v>
+        <v>0.001818992614523211</v>
       </c>
       <c r="E53" t="n">
-        <v>0.5588247816793755</v>
+        <v>0.5555300293986313</v>
       </c>
       <c r="F53" t="n">
-        <v>174.9413600651272</v>
+        <v>174.8034918539843</v>
       </c>
     </row>
     <row r="54">
       <c r="C54" t="n">
-        <v>57.90443980602486</v>
+        <v>17.06407375255261</v>
       </c>
       <c r="D54" t="n">
-        <v>7.737245091594671e-11</v>
+        <v>0.001155957709954221</v>
       </c>
       <c r="E54" t="n">
-        <v>0.5588247825431738</v>
+        <v>0.5568777242352784</v>
       </c>
       <c r="F54" t="n">
-        <v>174.9413600961263</v>
+        <v>174.965756619213</v>
       </c>
     </row>
     <row r="55">
       <c r="C55" t="n">
-        <v>62.60516572014821</v>
+        <v>18.02090586049144</v>
       </c>
       <c r="D55" t="n">
-        <v>1.780127252603834e-11</v>
+        <v>0.0007169692375951795</v>
       </c>
       <c r="E55" t="n">
-        <v>0.5588247827668666</v>
+        <v>0.557773762554898</v>
       </c>
       <c r="F55" t="n">
-        <v>174.9413601035512</v>
+        <v>175.0679129641221</v>
       </c>
     </row>
     <row r="56">
       <c r="C56" t="n">
-        <v>67.68750009458535</v>
+        <v>19.03139031991789</v>
       </c>
       <c r="D56" t="n">
-        <v>3.896876552631625e-12</v>
+        <v>0.0004340169236544989</v>
       </c>
       <c r="E56" t="n">
-        <v>0.5588247828220053</v>
+        <v>0.5583552893693768</v>
       </c>
       <c r="F56" t="n">
-        <v>174.941360105244</v>
+        <v>175.1306919953214</v>
       </c>
     </row>
     <row r="57">
       <c r="C57" t="n">
-        <v>73.18242219076174</v>
+        <v>20.09853557379314</v>
       </c>
       <c r="D57" t="n">
-        <v>8.116768353647595e-13</v>
+        <v>0.0002564250048837759</v>
       </c>
       <c r="E57" t="n">
-        <v>0.5588247828349419</v>
+        <v>0.5587236902829349</v>
       </c>
       <c r="F57" t="n">
-        <v>174.9413601056113</v>
+        <v>175.1683512451302</v>
       </c>
     </row>
     <row r="58">
       <c r="C58" t="n">
-        <v>79.12342618981323</v>
+        <v>21.22551875720087</v>
       </c>
       <c r="D58" t="n">
-        <v>1.608609242079827e-13</v>
+        <v>0.0001478637262860358</v>
       </c>
       <c r="E58" t="n">
-        <v>0.5588247828378308</v>
+        <v>0.5589515035835697</v>
       </c>
       <c r="F58" t="n">
-        <v>174.9413601056872</v>
+        <v>175.1904026439412</v>
       </c>
     </row>
     <row r="59">
       <c r="C59" t="n">
-        <v>85.5467253556568</v>
+        <v>22.41569515640389</v>
       </c>
       <c r="D59" t="n">
-        <v>3.033324491973887e-14</v>
+        <v>8.321669943047392e-05</v>
       </c>
       <c r="E59" t="n">
-        <v>0.5588247828384448</v>
+        <v>0.5590890168180725</v>
       </c>
       <c r="F59" t="n">
-        <v>174.9413601057021</v>
+        <v>175.2030066228108</v>
       </c>
     </row>
     <row r="60">
       <c r="C60" t="n">
-        <v>92.49147277217335</v>
+        <v>23.6726081982974</v>
       </c>
       <c r="D60" t="n">
-        <v>5.442370304116776e-15</v>
+        <v>4.570954441547913e-05</v>
       </c>
       <c r="E60" t="n">
-        <v>0.5588247828385691</v>
+        <v>0.5591700413567388</v>
       </c>
       <c r="F60" t="n">
-        <v>174.9413601057049</v>
+        <v>175.2100387357565</v>
       </c>
     </row>
     <row r="61">
       <c r="C61" t="n">
-        <v>100</v>
+        <v>25.00000000000001</v>
       </c>
       <c r="D61" t="n">
-        <v>9.290909058257823e-16</v>
+        <v>2.450478321149864e-05</v>
       </c>
       <c r="E61" t="n">
-        <v>0.5588247828385929</v>
+        <v>0.5592166423181658</v>
       </c>
       <c r="F61" t="n">
-        <v>174.9413601057054</v>
+        <v>175.2138684842045</v>
       </c>
     </row>
   </sheetData>
@@ -2556,7 +2556,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>40.66198599282025</v>
+        <v>40.72571625306137</v>
       </c>
     </row>
     <row r="6">
@@ -2566,7 +2566,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>177.0016250267465</v>
+        <v>177.2790428495761</v>
       </c>
     </row>
     <row r="7">
@@ -2586,7 +2586,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.5588247828385928</v>
+        <v>0.5592166423181656</v>
       </c>
     </row>
     <row r="9">
@@ -2596,7 +2596,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>12.77741941644749</v>
+        <v>12.76649267905592</v>
       </c>
     </row>
     <row r="10">
@@ -2606,7 +2606,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>6.02089449333613</v>
+        <v>6.05199623145259</v>
       </c>
     </row>
     <row r="11">
@@ -2616,7 +2616,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>174.9413601057054</v>
+        <v>175.2138684842045</v>
       </c>
     </row>
     <row r="12">
@@ -2626,7 +2626,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.5588247828385929</v>
+        <v>0.5592166423181658</v>
       </c>
     </row>
   </sheetData>

</xml_diff>